<commit_message>
Continue working on Smoke Test Cases Implementation + Exploratory Test Case Creation
</commit_message>
<xml_diff>
--- a/E-Commerce Web/Amazon/Test Suites/Functional Testing Suite/Exploratory Tests.xlsx
+++ b/E-Commerce Web/Amazon/Test Suites/Functional Testing Suite/Exploratory Tests.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -36,25 +36,52 @@
     <t>Test Case Description</t>
   </si>
   <si>
-    <t>Test Case Steps</t>
-  </si>
-  <si>
-    <t>Expected Result</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
     <t>Comments</t>
   </si>
   <si>
-    <t>1.</t>
-  </si>
-  <si>
-    <t>2.</t>
-  </si>
-  <si>
-    <t>3.</t>
+    <t>TC-EXP-1</t>
+  </si>
+  <si>
+    <t>Session 1</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>1. Enter the Amazon Page</t>
+  </si>
+  <si>
+    <t>Status (Mobile)</t>
+  </si>
+  <si>
+    <t>TC-EXP-2</t>
+  </si>
+  <si>
+    <t>TC-EXP-3</t>
+  </si>
+  <si>
+    <t>Session 2</t>
+  </si>
+  <si>
+    <t>Session 3</t>
+  </si>
+  <si>
+    <t>1. Enter the Amazon Page           2. Choose a department (Baby)</t>
+  </si>
+  <si>
+    <t>Just explore the application for next 30 minutes</t>
+  </si>
+  <si>
+    <t>Just explore the application for next 45 minutes in the exact department</t>
+  </si>
+  <si>
+    <t>Just explore the application (Your Account) for next 15 minutes</t>
+  </si>
+  <si>
+    <t>1. Enter the Amazon Page           2. Go to (All -&gt; Your Account)</t>
   </si>
 </sst>
 </file>
@@ -142,22 +169,36 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -438,87 +479,191 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:J5"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.109375" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="13.21875" customWidth="1"/>
+    <col min="4" max="4" width="26.6640625" customWidth="1"/>
+    <col min="5" max="5" width="31.21875" customWidth="1"/>
+    <col min="6" max="6" width="6.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13" customWidth="1"/>
+    <col min="8" max="8" width="10.88671875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B2" s="1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="1" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-    </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="D2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="4"/>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="4"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="4"/>
-      <c r="G4" s="1" t="s">
-        <v>10</v>
-      </c>
+      <c r="G4" s="4"/>
       <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-    </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="I3:I5"/>
-    <mergeCell ref="J3:J5"/>
-    <mergeCell ref="B3:B5"/>
-    <mergeCell ref="C3:C5"/>
-    <mergeCell ref="D3:D5"/>
-    <mergeCell ref="E3:E5"/>
-    <mergeCell ref="F3:F5"/>
-    <mergeCell ref="H3:H5"/>
+  <mergeCells count="24">
+    <mergeCell ref="H8:H10"/>
+    <mergeCell ref="F2:F4"/>
+    <mergeCell ref="G2:G4"/>
+    <mergeCell ref="G5:G7"/>
+    <mergeCell ref="F5:F7"/>
+    <mergeCell ref="F8:F10"/>
+    <mergeCell ref="G8:G10"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="E8:E10"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="D2:D4"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="H2:H4"/>
+    <mergeCell ref="H5:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Finalized Implementation of Smoke & Exploratory Testing
</commit_message>
<xml_diff>
--- a/E-Commerce Web/Amazon/Test Suites/Functional Testing Suite/Exploratory Tests.xlsx
+++ b/E-Commerce Web/Amazon/Test Suites/Functional Testing Suite/Exploratory Tests.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="23">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -82,6 +82,12 @@
   </si>
   <si>
     <t>1. Enter the Amazon Page           2. Go to (All -&gt; Your Account)</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>Some products do not satisfy the "Baby" department logically</t>
   </si>
 </sst>
 </file>
@@ -182,6 +188,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -189,15 +204,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -489,7 +495,7 @@
     <col min="5" max="5" width="31.21875" customWidth="1"/>
     <col min="6" max="6" width="6.33203125" customWidth="1"/>
     <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="10.88671875" customWidth="1"/>
+    <col min="8" max="8" width="26.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -528,22 +534,26 @@
       <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
+      <c r="F2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="H2" s="2"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="6"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
@@ -552,8 +562,8 @@
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="7"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -568,35 +578,41 @@
       <c r="C5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
+      <c r="F5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
+      <c r="H6" s="6"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
+      <c r="H7" s="7"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
@@ -608,22 +624,26 @@
       <c r="C8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
+      <c r="F8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="H8" s="2"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
@@ -632,14 +652,29 @@
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="D2:D4"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="E8:E10"/>
     <mergeCell ref="H8:H10"/>
     <mergeCell ref="F2:F4"/>
     <mergeCell ref="G2:G4"/>
@@ -647,21 +682,6 @@
     <mergeCell ref="F5:F7"/>
     <mergeCell ref="F8:F10"/>
     <mergeCell ref="G8:G10"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="D8:D10"/>
-    <mergeCell ref="E8:E10"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="C5:C7"/>
-    <mergeCell ref="D5:D7"/>
-    <mergeCell ref="E5:E7"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="C2:C4"/>
-    <mergeCell ref="D2:D4"/>
-    <mergeCell ref="E2:E4"/>
     <mergeCell ref="H2:H4"/>
     <mergeCell ref="H5:H7"/>
   </mergeCells>

</xml_diff>